<commit_message>
fix: parking json format
</commit_message>
<xml_diff>
--- a/python-src/venues.xlsx
+++ b/python-src/venues.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:D55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,23 +432,987 @@
           <t>handler</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>location</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>Ariana Grande Oakland</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/parking-passes-only-ariana-grande-oakland-tickets-6-6-2026/event/159278587/</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Oakland, CA</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Hatsune Miku</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/hatsune-miku-tickets/performer/1495258?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Joe Hisaishi</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/joe-hisaishi-tickets/performer/100313518?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Just In Time</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/just-in-time-tickets/performer/150427956?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Les Miserables The Arena Spectacular</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/les-miserables-the-arena-spectacular-tickets/performer/150342671?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Moulin Rouge The Musical</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/moulin-rouge-the-musical-tickets/performer/150374069?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>New Jersey Devils</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/new-jersey-devils-tickets/performer/3023?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>New York City Fc</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/new-york-city-fc-tickets/performer/1495038?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>New York Knicks</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/new-york-knicks-tickets/performer/2742?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>New York Liberty</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/new-york-liberty-tickets/performer/13974?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>New York Yankees</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/new-york-yankees-tickets/performer/5650?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Oh Mary</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/oh-mary-tickets/performer/150204986?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Savannah Bananas</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/savannah-bananas-tickets/performer/100283621?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Stars On Ice</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/stars-on-ice-tickets/performer/9682?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Stranger Things The First Shadow</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/stranger-things-the-first-shadow-tickets/performer/150063590?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Wicked The Musical</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/wicked-the-musical-tickets/performer/150289950?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Akaash Singh</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/akaash-singh-tickets/performer/102016768?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Aladdin The Musical</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/aladdin-the-musical-tickets/performer/170487?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
           <t>Ariana Grande</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>https://www.stubhub.com/ariana-grande-tickets/performer/511927?gridFilterType=1</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>stubhub-discovery</t>
-        </is>
-      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Bert Kreischer</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/bert-kreischer-tickets/performer/1514654?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Blue Man Group</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/blue-man-group-tickets/performer/43488?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Bon Jovi</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/bon-jovi-tickets/performer/916?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Bruce Springsteen</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/bruce-springsteen-tickets/performer/5984?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Bruno Mars</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/bruno-mars-tickets/performer/492103?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Bts</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/bts-tickets/performer/1503185?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Carin Leon</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/carin-leon-tickets/performer/100326849?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Chris Stapleton</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/chris-stapleton-tickets/performer/1493916?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ed Sheeran</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/ed-sheeran-tickets/performer/700045?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Five Finger Death Punch</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/five-finger-death-punch-tickets/performer/339237?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Gabriel Iglesias</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/gabriel-iglesias-tickets/performer/223487?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Harry Styles</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/harry-styles-tickets/performer/1521417?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>J Cole</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/j-cole-tickets/performer/489774?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Jeff Arcuri</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/jeff-arcuri-tickets/performer/100270259?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Jerry Seinfeld</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/jerry-seinfeld-tickets/performer/984?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Jim Gaffigan</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/jim-gaffigan-tickets/performer/98417?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Jo Koy</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/jo-koy-tickets/performer/405174?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>John Oliver</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/john-oliver-tickets/performer/367490?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Lady Gaga</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/lady-gaga-tickets/performer/374244?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Martin Lawrence</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/martin-lawrence-tickets/performer/3503?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Michael Mcintyre</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/michael-mcintyre-tickets/performer/700088?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Michelle Buteau</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/michelle-buteau-tickets/performer/729045?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Nate Bargatze</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/nate-bargatze-tickets/performer/100269979?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Nimesh Patel</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/nimesh-patel-tickets/performer/101883460?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Noah Kahan</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/noah-kahan-tickets/performer/100276660?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Olivia Dean</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/olivia-dean-tickets/performer/138291382?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Ringling Bros And Barnum And Bailey Circus</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/ringling-bros-and-barnum-and-bailey-circus-tickets/performer/134724?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Rush</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/rush-tickets/performer/5324?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Russell Peters</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/russell-peters-tickets/performer/130925?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Sarah Mclachlan</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/sarah-mclachlan-tickets/performer/9921?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Tim Dillon</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/tim-dillon-tickets/performer/100270258?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Weird Al Yankovic</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/weird-al-yankovic-tickets/performer/11047?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Whiskey Myers</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/whiskey-myers-tickets/performer/1494397?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Ye</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/ye-tickets/performer/30290?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Yunchan Lim</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://www.stubhub.com/yunchan-lim-tickets/performer/150017608?gridFilterType=1</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>stubhub-discovery</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
fix:forced USD only and excel for phase 2
</commit_message>
<xml_diff>
--- a/python-src/venues.xlsx
+++ b/python-src/venues.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:D54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,12 +441,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Ariana Grande Oakland</t>
+          <t>Akaash Singh</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/parking-passes-only-ariana-grande-oakland-tickets-6-6-2026/event/159278587/</t>
+          <t>https://www.stubhub.com/akaash-singh-tickets/performer/102016768?gridFilterType=1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -454,21 +454,17 @@
           <t>stubhub-discovery</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Oakland, CA</t>
-        </is>
-      </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hatsune Miku</t>
+          <t>Aladdin The Musical</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/hatsune-miku-tickets/performer/1495258?gridFilterType=1</t>
+          <t>https://www.stubhub.com/aladdin-the-musical-tickets/performer/170487?gridFilterType=1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -481,12 +477,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Joe Hisaishi</t>
+          <t>Ariana Grande</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/joe-hisaishi-tickets/performer/100313518?gridFilterType=1</t>
+          <t>https://www.stubhub.com/ariana-grande-tickets/performer/511927?gridFilterType=1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -499,12 +495,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Just In Time</t>
+          <t>Bert Kreischer</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/just-in-time-tickets/performer/150427956?gridFilterType=1</t>
+          <t>https://www.stubhub.com/bert-kreischer-tickets/performer/1514654?gridFilterType=1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -517,12 +513,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Les Miserables The Arena Spectacular</t>
+          <t>Bon Jovi</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/les-miserables-the-arena-spectacular-tickets/performer/150342671?gridFilterType=1</t>
+          <t>https://www.stubhub.com/bon-jovi-tickets/performer/916?gridFilterType=1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -535,12 +531,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Moulin Rouge The Musical</t>
+          <t>Bruce Springsteen</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/moulin-rouge-the-musical-tickets/performer/150374069?gridFilterType=1</t>
+          <t>https://www.stubhub.com/bruce-springsteen-tickets/performer/5984?gridFilterType=1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -553,12 +549,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>New Jersey Devils</t>
+          <t>Bruno Mars</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/new-jersey-devils-tickets/performer/3023?gridFilterType=1</t>
+          <t>https://www.stubhub.com/bruno-mars-tickets/performer/492103?gridFilterType=1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -571,12 +567,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>New York City Fc</t>
+          <t>Bts</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/new-york-city-fc-tickets/performer/1495038?gridFilterType=1</t>
+          <t>https://www.stubhub.com/bts-tickets/performer/1503185?gridFilterType=1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -589,12 +585,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>New York Knicks</t>
+          <t>Carin Leon</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/new-york-knicks-tickets/performer/2742?gridFilterType=1</t>
+          <t>https://www.stubhub.com/carin-leon-tickets/performer/100326849?gridFilterType=1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -607,12 +603,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>New York Liberty</t>
+          <t>Chris Stapleton</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/new-york-liberty-tickets/performer/13974?gridFilterType=1</t>
+          <t>https://www.stubhub.com/chris-stapleton-tickets/performer/1493916?gridFilterType=1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -625,12 +621,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>New York Yankees</t>
+          <t>Ed Sheeran</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/new-york-yankees-tickets/performer/5650?gridFilterType=1</t>
+          <t>https://www.stubhub.com/ed-sheeran-tickets/performer/700045?gridFilterType=1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -643,12 +639,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Oh Mary</t>
+          <t>Five Finger Death Punch</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/oh-mary-tickets/performer/150204986?gridFilterType=1</t>
+          <t>https://www.stubhub.com/five-finger-death-punch-tickets/performer/339237?gridFilterType=1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -661,12 +657,12 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Savannah Bananas</t>
+          <t>Gabriel Iglesias</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/savannah-bananas-tickets/performer/100283621?gridFilterType=1</t>
+          <t>https://www.stubhub.com/gabriel-iglesias-tickets/performer/223487?gridFilterType=1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -679,12 +675,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Stars On Ice</t>
+          <t>Harry Styles</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/stars-on-ice-tickets/performer/9682?gridFilterType=1</t>
+          <t>https://www.stubhub.com/harry-styles-tickets/performer/1521417?gridFilterType=1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -697,12 +693,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stranger Things The First Shadow</t>
+          <t>Hatsune Miku</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/stranger-things-the-first-shadow-tickets/performer/150063590?gridFilterType=1</t>
+          <t>https://www.stubhub.com/hatsune-miku-tickets/performer/1495258?gridFilterType=1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -715,12 +711,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Wicked The Musical</t>
+          <t>Jeff Arcuri</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/wicked-the-musical-tickets/performer/150289950?gridFilterType=1</t>
+          <t>https://www.stubhub.com/jeff-arcuri-tickets/performer/100270259?gridFilterType=1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -733,12 +729,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Akaash Singh</t>
+          <t>Jerry Seinfeld</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/akaash-singh-tickets/performer/102016768?gridFilterType=1</t>
+          <t>https://www.stubhub.com/jerry-seinfeld-tickets/performer/984?gridFilterType=1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -751,12 +747,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Aladdin The Musical</t>
+          <t>Jim Gaffigan</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/aladdin-the-musical-tickets/performer/170487?gridFilterType=1</t>
+          <t>https://www.stubhub.com/jim-gaffigan-tickets/performer/98417?gridFilterType=1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -769,12 +765,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Ariana Grande</t>
+          <t>Jo Koy</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/ariana-grande-tickets/performer/511927?gridFilterType=1</t>
+          <t>https://www.stubhub.com/jo-koy-tickets/performer/405174?gridFilterType=1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -787,12 +783,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Bert Kreischer</t>
+          <t>Joe Hisaishi</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/bert-kreischer-tickets/performer/1514654?gridFilterType=1</t>
+          <t>https://www.stubhub.com/joe-hisaishi-tickets/performer/100313518?gridFilterType=1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -805,12 +801,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Blue Man Group</t>
+          <t>John Oliver</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/blue-man-group-tickets/performer/43488?gridFilterType=1</t>
+          <t>https://www.stubhub.com/john-oliver-tickets/performer/367490?gridFilterType=1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -823,12 +819,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Bon Jovi</t>
+          <t>Just In Time</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/bon-jovi-tickets/performer/916?gridFilterType=1</t>
+          <t>https://www.stubhub.com/just-in-time-tickets/performer/150427956?gridFilterType=1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -841,12 +837,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Bruce Springsteen</t>
+          <t>Lady Gaga</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/bruce-springsteen-tickets/performer/5984?gridFilterType=1</t>
+          <t>https://www.stubhub.com/lady-gaga-tickets/performer/374244?gridFilterType=1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -859,12 +855,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Bruno Mars</t>
+          <t>Les Miserables The Arena Spectacular</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/bruno-mars-tickets/performer/492103?gridFilterType=1</t>
+          <t>https://www.stubhub.com/les-miserables-the-arena-spectacular-tickets/performer/150342671?gridFilterType=1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -877,12 +873,12 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Bts</t>
+          <t>Lionel Richie</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/bts-tickets/performer/1503185?gridFilterType=1</t>
+          <t>https://www.stubhub.com/lionel-richie-tickets/performer/43889?gridFilterType=1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -895,12 +891,12 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Carin Leon</t>
+          <t>Liverpool Fc</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/carin-leon-tickets/performer/100326849?gridFilterType=1</t>
+          <t>https://www.stubhub.com/liverpool-fc-tickets/performer/13327?gridFilterType=1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -913,12 +909,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Chris Stapleton</t>
+          <t>Metallica</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/chris-stapleton-tickets/performer/1493916?gridFilterType=1</t>
+          <t>https://www.stubhub.com/metallica-tickets/performer/8147?gridFilterType=1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -931,12 +927,12 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Ed Sheeran</t>
+          <t>Michael Mcintyre</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/ed-sheeran-tickets/performer/700045?gridFilterType=1</t>
+          <t>https://www.stubhub.com/michael-mcintyre-tickets/performer/700088?gridFilterType=1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -949,12 +945,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Five Finger Death Punch</t>
+          <t>Michelle Buteau</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/five-finger-death-punch-tickets/performer/339237?gridFilterType=1</t>
+          <t>https://www.stubhub.com/michelle-buteau-tickets/performer/729045?gridFilterType=1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -967,12 +963,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Gabriel Iglesias</t>
+          <t>Moulin Rouge The Musical</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/gabriel-iglesias-tickets/performer/223487?gridFilterType=1</t>
+          <t>https://www.stubhub.com/moulin-rouge-the-musical-tickets/performer/150374069?gridFilterType=1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -985,12 +981,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Harry Styles</t>
+          <t>Nate Bargatze</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/harry-styles-tickets/performer/1521417?gridFilterType=1</t>
+          <t>https://www.stubhub.com/nate-bargatze-tickets/performer/100269979?gridFilterType=1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1003,12 +999,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>J Cole</t>
+          <t>New Jersey Devils</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/j-cole-tickets/performer/489774?gridFilterType=1</t>
+          <t>https://www.stubhub.com/new-jersey-devils-tickets/performer/3023?gridFilterType=1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1021,12 +1017,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Jeff Arcuri</t>
+          <t>New York City Fc</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/jeff-arcuri-tickets/performer/100270259?gridFilterType=1</t>
+          <t>https://www.stubhub.com/new-york-city-fc-tickets/performer/1495038?gridFilterType=1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1039,12 +1035,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Jerry Seinfeld</t>
+          <t>New York Knicks</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/jerry-seinfeld-tickets/performer/984?gridFilterType=1</t>
+          <t>https://www.stubhub.com/new-york-knicks-tickets/performer/2742?gridFilterType=1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1057,12 +1053,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Jim Gaffigan</t>
+          <t>New York Liberty</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/jim-gaffigan-tickets/performer/98417?gridFilterType=1</t>
+          <t>https://www.stubhub.com/new-york-liberty-tickets/performer/13974?gridFilterType=1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1075,12 +1071,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Jo Koy</t>
+          <t>New York Yankees</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/jo-koy-tickets/performer/405174?gridFilterType=1</t>
+          <t>https://www.stubhub.com/new-york-yankees-tickets/performer/5650?gridFilterType=1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1093,12 +1089,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>John Oliver</t>
+          <t>Nimesh Patel</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/john-oliver-tickets/performer/367490?gridFilterType=1</t>
+          <t>https://www.stubhub.com/nimesh-patel-tickets/performer/101883460?gridFilterType=1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1111,12 +1107,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Lady Gaga</t>
+          <t>Noah Kahan</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/lady-gaga-tickets/performer/374244?gridFilterType=1</t>
+          <t>https://www.stubhub.com/noah-kahan-tickets/performer/100276660?gridFilterType=1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1129,12 +1125,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Martin Lawrence</t>
+          <t>Oh Mary</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/martin-lawrence-tickets/performer/3503?gridFilterType=1</t>
+          <t>https://www.stubhub.com/oh-mary-tickets/performer/150204986?gridFilterType=1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1147,12 +1143,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Michael Mcintyre</t>
+          <t>Olivia Dean</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/michael-mcintyre-tickets/performer/700088?gridFilterType=1</t>
+          <t>https://www.stubhub.com/olivia-dean-tickets/performer/138291382?gridFilterType=1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1165,12 +1161,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Michelle Buteau</t>
+          <t>Ringling Bros And Barnum And Bailey Circus</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/michelle-buteau-tickets/performer/729045?gridFilterType=1</t>
+          <t>https://www.stubhub.com/ringling-bros-and-barnum-and-bailey-circus-tickets/performer/134724?gridFilterType=1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1183,12 +1179,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Nate Bargatze</t>
+          <t>Rush</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/nate-bargatze-tickets/performer/100269979?gridFilterType=1</t>
+          <t>https://www.stubhub.com/rush-tickets/performer/5324?gridFilterType=1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1201,12 +1197,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Nimesh Patel</t>
+          <t>Russell Peters</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/nimesh-patel-tickets/performer/101883460?gridFilterType=1</t>
+          <t>https://www.stubhub.com/russell-peters-tickets/performer/130925?gridFilterType=1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1219,12 +1215,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Noah Kahan</t>
+          <t>Sarah Mclachlan</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/noah-kahan-tickets/performer/100276660?gridFilterType=1</t>
+          <t>https://www.stubhub.com/sarah-mclachlan-tickets/performer/9921?gridFilterType=1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1237,12 +1233,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Olivia Dean</t>
+          <t>Savannah Bananas</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/olivia-dean-tickets/performer/138291382?gridFilterType=1</t>
+          <t>https://www.stubhub.com/savannah-bananas-tickets/performer/100283621?gridFilterType=1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1255,12 +1251,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Ringling Bros And Barnum And Bailey Circus</t>
+          <t>Sebastian Maniscalco</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/ringling-bros-and-barnum-and-bailey-circus-tickets/performer/134724?gridFilterType=1</t>
+          <t>https://www.stubhub.com/sebastian-maniscalco-tickets/performer/492595?gridFilterType=1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1273,12 +1269,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Rush</t>
+          <t>Six The Musical</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/rush-tickets/performer/5324?gridFilterType=1</t>
+          <t>https://www.stubhub.com/six-the-musical-tickets/performer/150328705?gridFilterType=1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -1291,12 +1287,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Russell Peters</t>
+          <t>Stars On Ice</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/russell-peters-tickets/performer/130925?gridFilterType=1</t>
+          <t>https://www.stubhub.com/stars-on-ice-tickets/performer/9682?gridFilterType=1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1309,12 +1305,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Sarah Mclachlan</t>
+          <t>Stranger Things The First Shadow</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/sarah-mclachlan-tickets/performer/9921?gridFilterType=1</t>
+          <t>https://www.stubhub.com/stranger-things-the-first-shadow-tickets/performer/150063590?gridFilterType=1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1363,12 +1359,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Whiskey Myers</t>
+          <t>Wicked The Musical</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/whiskey-myers-tickets/performer/1494397?gridFilterType=1</t>
+          <t>https://www.stubhub.com/wicked-the-musical-tickets/performer/150289950?gridFilterType=1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1381,12 +1377,12 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Ye</t>
+          <t>Yunchan Lim</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>https://www.stubhub.com/ye-tickets/performer/30290?gridFilterType=1</t>
+          <t>https://www.stubhub.com/yunchan-lim-tickets/performer/150017608?gridFilterType=1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1395,24 +1391,6 @@
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Yunchan Lim</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>https://www.stubhub.com/yunchan-lim-tickets/performer/150017608?gridFilterType=1</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>stubhub-discovery</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>